<commit_message>
fix(audit): 對齊 workbook semantic-key index 與 fixture 契約
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/audit/sample_workbook.xlsx
+++ b/tests/fixtures/audit/sample_workbook.xlsx
@@ -413,150 +413,308 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Topology</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Object</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Command Output</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
         <is>
           <t>5G</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>6G</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>2.4G</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Device .1.</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>DoThing</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>step1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>out1</t>
-        </is>
-      </c>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>Noise</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>WiFi.Radio.{i}.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>ubus-cli WiFi.Radio.1.Noise?</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>expected</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Device .1.</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>DoThing</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>step2</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>out2</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SRGBSSColorBitmap</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>WiFi.Radio.{i}.IEEE80211ax.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>ubus-cli set + grep hostapd.conf</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>see source</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>OtherDevice.</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>OtherAPI</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
-      </c>
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>DuplicateApi</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>WiFi.Radio.{i}.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>first occurrence</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DuplicateApi</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>WiFi.Radio.{i}.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>second occurrence</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
     </row>

</xml_diff>